<commit_message>
Sidebar dropdown with techno-economic model inputs for each technology
Loading of general information from excel and CAPEX/OPEX tables per technology from excel model files. Structure and naming conventions of the base template.
</commit_message>
<xml_diff>
--- a/backend/design-capital-structure/design-capital-structure-Aligned.xlsx
+++ b/backend/design-capital-structure/design-capital-structure-Aligned.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="JUST ACCESS" sheetId="1" state="visible" r:id="rId1"/>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0\ &quot;M$&quot;;\ \(#,##0\)\ &quot;M$&quot;;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -107,9 +107,6 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -143,7 +140,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -177,18 +174,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -239,9 +230,6 @@
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -827,7 +815,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -931,7 +919,7 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -1167,7 +1155,7 @@
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -1413,7 +1401,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1525,7 +1513,7 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
@@ -1773,7 +1761,7 @@
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Units</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -2033,493 +2021,587 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr codeName="Hoja3">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="39.36328125" customWidth="1" min="1" max="1"/>
+    <col width="24.6328125" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Financiation</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="C1" s="17" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="D1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 3</t>
-        </is>
-      </c>
-      <c r="E1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 4</t>
-        </is>
-      </c>
-      <c r="F1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 8</t>
-        </is>
-      </c>
-      <c r="G1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 9</t>
-        </is>
-      </c>
-      <c r="H1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 10</t>
-        </is>
-      </c>
-      <c r="I1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 11</t>
-        </is>
-      </c>
-      <c r="J1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 12</t>
-        </is>
-      </c>
-      <c r="K1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 13</t>
-        </is>
-      </c>
-      <c r="L1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 14</t>
-        </is>
-      </c>
-      <c r="M1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 15</t>
-        </is>
-      </c>
-      <c r="N1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 16</t>
-        </is>
-      </c>
-      <c r="O1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 17</t>
-        </is>
-      </c>
-      <c r="P1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 18</t>
-        </is>
-      </c>
-      <c r="Q1" s="17" t="inlineStr">
-        <is>
-          <t>Unnamed: 19</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>How much to be finance (till 2034)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>M$</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="C2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>How much to be finance (till 2030 - SDG 7 targets)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>M$</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="C3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
+      <c r="P3" s="1" t="n"/>
+      <c r="Q3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="1" t="n"/>
+      <c r="K4" s="1" t="n"/>
+      <c r="L4" s="1" t="n"/>
+      <c r="M4" s="1" t="n"/>
+      <c r="N4" s="1" t="n"/>
+      <c r="O4" s="1" t="n"/>
+      <c r="P4" s="1" t="n"/>
+      <c r="Q4" s="1" t="n"/>
+    </row>
+    <row r="5" ht="15" customHeight="1" thickBot="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Total </t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Amount Total</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Amount Division</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="F5" s="1" t="n"/>
+      <c r="G5" s="1" t="n"/>
+      <c r="H5" s="1" t="n"/>
+      <c r="I5" s="1" t="n"/>
+      <c r="J5" s="1" t="n"/>
+      <c r="K5" s="1" t="n"/>
+      <c r="L5" s="1" t="n"/>
+      <c r="M5" s="1" t="n"/>
+      <c r="N5" s="1" t="n"/>
+      <c r="O5" s="1" t="n"/>
+      <c r="P5" s="1" t="n"/>
+      <c r="Q5" s="1" t="n"/>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Total:</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="B6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>1.- Equity (to be injected in year 0)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="E6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="1" t="n"/>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="n"/>
+      <c r="O6" s="1" t="n"/>
+      <c r="P6" s="1" t="n"/>
+      <c r="Q6" s="1" t="n"/>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Total:</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>2.- Grants (inyected in the first two years but linked to CAPEX deployment)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="E7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1" t="n"/>
+      <c r="G7" s="1" t="n"/>
+      <c r="H7" s="1" t="n"/>
+      <c r="I7" s="1" t="n"/>
+      <c r="J7" s="1" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="1" t="n"/>
+      <c r="M7" s="1" t="n"/>
+      <c r="N7" s="1" t="n"/>
+      <c r="O7" s="1" t="n"/>
+      <c r="P7" s="1" t="n"/>
+      <c r="Q7" s="1" t="n"/>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Total:</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>3.- Debt</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="C9" t="inlineStr">
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="n"/>
+      <c r="H8" s="1" t="n"/>
+      <c r="I8" s="1" t="n"/>
+      <c r="J8" s="1" t="n"/>
+      <c r="K8" s="1" t="n"/>
+      <c r="L8" s="1" t="n"/>
+      <c r="M8" s="1" t="n"/>
+      <c r="N8" s="1" t="n"/>
+      <c r="O8" s="1" t="n"/>
+      <c r="P8" s="1" t="n"/>
+      <c r="Q8" s="1" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Interests</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="C10" t="inlineStr">
+      <c r="E9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1" t="n"/>
+      <c r="G9" s="1" t="n"/>
+      <c r="H9" s="1" t="n"/>
+      <c r="I9" s="1" t="n"/>
+      <c r="J9" s="1" t="n"/>
+      <c r="K9" s="1" t="n"/>
+      <c r="L9" s="1" t="n"/>
+      <c r="M9" s="1" t="n"/>
+      <c r="N9" s="1" t="n"/>
+      <c r="O9" s="1" t="n"/>
+      <c r="P9" s="1" t="n"/>
+      <c r="Q9" s="1" t="n"/>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Grace period</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="C11" t="inlineStr">
+      <c r="E10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="n"/>
+      <c r="H10" s="1" t="n"/>
+      <c r="I10" s="1" t="n"/>
+      <c r="J10" s="1" t="n"/>
+      <c r="K10" s="1" t="n"/>
+      <c r="L10" s="1" t="n"/>
+      <c r="M10" s="1" t="n"/>
+      <c r="N10" s="1" t="n"/>
+      <c r="O10" s="1" t="n"/>
+      <c r="P10" s="1" t="n"/>
+      <c r="Q10" s="1" t="n"/>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Amortization period</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12"/>
+      <c r="E11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
+      <c r="H11" s="1" t="n"/>
+      <c r="I11" s="1" t="n"/>
+      <c r="J11" s="1" t="n"/>
+      <c r="K11" s="1" t="n"/>
+      <c r="L11" s="1" t="n"/>
+      <c r="M11" s="1" t="n"/>
+      <c r="N11" s="1" t="n"/>
+      <c r="O11" s="1" t="n"/>
+      <c r="P11" s="1" t="n"/>
+      <c r="Q11" s="1" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
+      <c r="H12" s="1" t="n"/>
+      <c r="I12" s="1" t="n"/>
+      <c r="J12" s="1" t="n"/>
+      <c r="K12" s="1" t="n"/>
+      <c r="L12" s="1" t="n"/>
+      <c r="M12" s="1" t="n"/>
+      <c r="N12" s="1" t="n"/>
+      <c r="O12" s="1" t="n"/>
+      <c r="P12" s="1" t="n"/>
+      <c r="Q12" s="1" t="n"/>
+    </row>
     <row r="13">
-      <c r="C13" t="inlineStr">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="9" t="n">
         <v>2023</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="9" t="n">
         <v>2024</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="9" t="n">
         <v>2025</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="9" t="n">
         <v>2026</v>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" s="9" t="n">
         <v>2027</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" s="9" t="n">
         <v>2028</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L13" s="9" t="n">
         <v>2029</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M13" s="9" t="n">
         <v>2030</v>
       </c>
-      <c r="N13" t="n">
+      <c r="N13" s="9" t="n">
         <v>2031</v>
       </c>
-      <c r="O13" t="n">
+      <c r="O13" s="9" t="n">
         <v>2032</v>
       </c>
-      <c r="P13" t="n">
+      <c r="P13" s="9" t="n">
         <v>2033</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="Q13" s="9" t="n">
         <v>2034</v>
       </c>
     </row>
-    <row r="14">
-      <c r="C14" t="inlineStr">
+    <row r="14" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="1" t="n"/>
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Annual debt needs</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>increase debt</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="C15" t="inlineStr">
+      <c r="D14" s="1" t="n"/>
+      <c r="E14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!F22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="F14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!F22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="G14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!G22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="H14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!H22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="I14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!I22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="J14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!J22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="K14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!K22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="L14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!L22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="M14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!M22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="N14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!N22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="O14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!O22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="P14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!P22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="Q14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!Q22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1" thickBot="1" thickTop="1">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>How much to increase</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>M$</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="C16" t="inlineStr">
+      <c r="E15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>Debt increase</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>M$</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
+      <c r="E16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="13" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <conditionalFormatting sqref="C14:AJ14">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
+      <formula>"increase debt"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
+      <formula>"ok"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restructuring of techno-economic model handling and design capital structiure sections
Renamed General Information to Fuel Market Information. Separated carbon market from other fuel markets for improved platform coherence.

Restructured techno-economic model management page. Models
now created by defining a name and year range, rather than uploading an Excel file.

Optionally, users can upload Excel files (e.g. Aligned.xlsm, CleanStep.xlsm) to update its techno-economic inputs.

Techno-economic input tables are now editable directly on the platform, with save and reset options, allowing updates even after uploading an Excel model.

Reorganized platform sections, splitting Electricity into E-Cooking and Electricity (Just Access) to match Excel distinctions.
</commit_message>
<xml_diff>
--- a/backend/design-capital-structure/design-capital-structure-Aligned.xlsx
+++ b/backend/design-capital-structure/design-capital-structure-Aligned.xlsx
@@ -3,10 +3,10 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="JUST ACCESS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="E-Cooking" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Electricity" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="LPG" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -796,593 +796,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Hoja1">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
-  <cols>
-    <col width="30.6328125" customWidth="1" min="1" max="1"/>
-    <col width="71.6328125" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Financiation</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>How much to be finance (till 2034)</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="n"/>
-      <c r="H2" s="1" t="n"/>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1" t="n"/>
-      <c r="L2" s="1" t="n"/>
-      <c r="M2" s="1" t="n"/>
-      <c r="N2" s="1" t="n"/>
-      <c r="O2" s="1" t="n"/>
-      <c r="P2" s="1" t="n"/>
-      <c r="Q2" s="1" t="n"/>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>How much to be finance (till 2030 - SDG 7 targets)</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="1" t="n"/>
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="n"/>
-      <c r="G3" s="1" t="n"/>
-      <c r="H3" s="1" t="n"/>
-      <c r="I3" s="1" t="n"/>
-      <c r="J3" s="1" t="n"/>
-      <c r="K3" s="1" t="n"/>
-      <c r="L3" s="1" t="n"/>
-      <c r="M3" s="1" t="n"/>
-      <c r="N3" s="1" t="n"/>
-      <c r="O3" s="1" t="n"/>
-      <c r="P3" s="1" t="n"/>
-      <c r="Q3" s="1" t="n"/>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="1" t="n"/>
-      <c r="D4" s="1" t="n"/>
-      <c r="E4" s="1" t="n"/>
-      <c r="F4" s="1" t="n"/>
-      <c r="G4" s="1" t="n"/>
-      <c r="H4" s="1" t="n"/>
-      <c r="I4" s="1" t="n"/>
-      <c r="J4" s="1" t="n"/>
-      <c r="K4" s="1" t="n"/>
-      <c r="L4" s="1" t="n"/>
-      <c r="M4" s="1" t="n"/>
-      <c r="N4" s="1" t="n"/>
-      <c r="O4" s="1" t="n"/>
-      <c r="P4" s="1" t="n"/>
-      <c r="Q4" s="1" t="n"/>
-    </row>
-    <row r="5" ht="15" customHeight="1" thickBot="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total </t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Amount Total</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>Division</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>Amount Division</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="n"/>
-      <c r="G5" s="1" t="n"/>
-      <c r="H5" s="1" t="n"/>
-      <c r="I5" s="1" t="n"/>
-      <c r="J5" s="1" t="n"/>
-      <c r="K5" s="1" t="n"/>
-      <c r="L5" s="1" t="n"/>
-      <c r="M5" s="1" t="n"/>
-      <c r="N5" s="1" t="n"/>
-      <c r="O5" s="1" t="n"/>
-      <c r="P5" s="1" t="n"/>
-      <c r="Q5" s="1" t="n"/>
-    </row>
-    <row r="6" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Total:</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>1.- Equity (to be injected in year 0)</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="1" t="n"/>
-      <c r="H6" s="1" t="n"/>
-      <c r="I6" s="1" t="n"/>
-      <c r="J6" s="1" t="n"/>
-      <c r="K6" s="7" t="n"/>
-      <c r="L6" s="1" t="n"/>
-      <c r="M6" s="1" t="n"/>
-      <c r="N6" s="1" t="n"/>
-      <c r="O6" s="1" t="n"/>
-      <c r="P6" s="1" t="n"/>
-      <c r="Q6" s="1" t="n"/>
-    </row>
-    <row r="7" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Total:</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>2.- Grants (inyected in the first two years but linked to CAPEX deployment)</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="1" t="n"/>
-      <c r="G7" s="1" t="n"/>
-      <c r="H7" s="1" t="n"/>
-      <c r="I7" s="1" t="n"/>
-      <c r="J7" s="1" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="1" t="n"/>
-      <c r="M7" s="1" t="n"/>
-      <c r="N7" s="1" t="n"/>
-      <c r="O7" s="1" t="n"/>
-      <c r="P7" s="1" t="n"/>
-      <c r="Q7" s="1" t="n"/>
-    </row>
-    <row r="8" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Total:</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>3.- Debt</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="1" t="n"/>
-      <c r="F8" s="1" t="n"/>
-      <c r="G8" s="1" t="n"/>
-      <c r="H8" s="1" t="n"/>
-      <c r="I8" s="1" t="n"/>
-      <c r="J8" s="1" t="n"/>
-      <c r="K8" s="1" t="n"/>
-      <c r="L8" s="1" t="n"/>
-      <c r="M8" s="1" t="n"/>
-      <c r="N8" s="1" t="n"/>
-      <c r="O8" s="1" t="n"/>
-      <c r="P8" s="1" t="n"/>
-      <c r="Q8" s="1" t="n"/>
-    </row>
-    <row r="9" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A9" s="1" t="n"/>
-      <c r="B9" s="1" t="n"/>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Interests</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="1" t="n"/>
-      <c r="G9" s="1" t="n"/>
-      <c r="H9" s="1" t="n"/>
-      <c r="I9" s="1" t="n"/>
-      <c r="J9" s="1" t="n"/>
-      <c r="K9" s="1" t="n"/>
-      <c r="L9" s="1" t="n"/>
-      <c r="M9" s="1" t="n"/>
-      <c r="N9" s="1" t="n"/>
-      <c r="O9" s="1" t="n"/>
-      <c r="P9" s="1" t="n"/>
-      <c r="Q9" s="1" t="n"/>
-    </row>
-    <row r="10" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A10" s="1" t="n"/>
-      <c r="B10" s="1" t="n"/>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Grace period</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="1" t="n"/>
-      <c r="G10" s="1" t="n"/>
-      <c r="H10" s="1" t="n"/>
-      <c r="I10" s="1" t="n"/>
-      <c r="J10" s="1" t="n"/>
-      <c r="K10" s="1" t="n"/>
-      <c r="L10" s="1" t="n"/>
-      <c r="M10" s="1" t="n"/>
-      <c r="N10" s="1" t="n"/>
-      <c r="O10" s="1" t="n"/>
-      <c r="P10" s="1" t="n"/>
-      <c r="Q10" s="1" t="n"/>
-    </row>
-    <row r="11" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A11" s="1" t="n"/>
-      <c r="B11" s="1" t="n"/>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Amortization period</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>years</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="1" t="n"/>
-      <c r="G11" s="1" t="n"/>
-      <c r="H11" s="1" t="n"/>
-      <c r="I11" s="1" t="n"/>
-      <c r="J11" s="1" t="n"/>
-      <c r="K11" s="1" t="n"/>
-      <c r="L11" s="1" t="n"/>
-      <c r="M11" s="1" t="n"/>
-      <c r="N11" s="1" t="n"/>
-      <c r="O11" s="1" t="n"/>
-      <c r="P11" s="1" t="n"/>
-      <c r="Q11" s="1" t="n"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="1" t="n"/>
-      <c r="B12" s="1" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="1" t="n"/>
-      <c r="F12" s="1" t="n"/>
-      <c r="G12" s="1" t="n"/>
-      <c r="H12" s="1" t="n"/>
-      <c r="I12" s="1" t="n"/>
-      <c r="J12" s="1" t="n"/>
-      <c r="K12" s="1" t="n"/>
-      <c r="L12" s="1" t="n"/>
-      <c r="M12" s="1" t="n"/>
-      <c r="N12" s="1" t="n"/>
-      <c r="O12" s="1" t="n"/>
-      <c r="P12" s="1" t="n"/>
-      <c r="Q12" s="1" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="1" t="n"/>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>2024</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <v>2025</v>
-      </c>
-      <c r="I13" s="9" t="n">
-        <v>2026</v>
-      </c>
-      <c r="J13" s="9" t="n">
-        <v>2027</v>
-      </c>
-      <c r="K13" s="9" t="n">
-        <v>2028</v>
-      </c>
-      <c r="L13" s="9" t="n">
-        <v>2029</v>
-      </c>
-      <c r="M13" s="9" t="n">
-        <v>2030</v>
-      </c>
-      <c r="N13" s="9" t="n">
-        <v>2031</v>
-      </c>
-      <c r="O13" s="9" t="n">
-        <v>2032</v>
-      </c>
-      <c r="P13" s="9" t="n">
-        <v>2033</v>
-      </c>
-      <c r="Q13" s="9" t="n">
-        <v>2034</v>
-      </c>
-    </row>
-    <row r="14" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="1" t="n"/>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>Annual debt needs</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="n"/>
-      <c r="E14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!F22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="F14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!F22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="G14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!G22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="H14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!H22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="I14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!I22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="J14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!J22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="K14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!K22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="L14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!L22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="M14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!M22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="N14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!N22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="O14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!O22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="P14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!P22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-      <c r="Q14" s="11">
-        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!Q22&gt;0,"ok","increase debt")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="1" t="n"/>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>How much to increase</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="16" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="1" t="n"/>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Debt increase</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>M$</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="C14:AJ14">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
-      <formula>"increase debt"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
-      <formula>"ok"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Hoja2">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2005,6 +1418,593 @@
     <row r="23">
       <c r="T23" s="14" t="n"/>
       <c r="U23" s="14" t="n"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C14:AJ14">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
+      <formula>"increase debt"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
+      <formula>"ok"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Hoja1">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="30.6328125" customWidth="1" min="1" max="1"/>
+    <col width="71.6328125" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Financiation</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>How much to be finance (till 2034)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>How much to be finance (till 2030 - SDG 7 targets)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
+      <c r="P3" s="1" t="n"/>
+      <c r="Q3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="1" t="n"/>
+      <c r="D4" s="1" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="1" t="n"/>
+      <c r="H4" s="1" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="1" t="n"/>
+      <c r="K4" s="1" t="n"/>
+      <c r="L4" s="1" t="n"/>
+      <c r="M4" s="1" t="n"/>
+      <c r="N4" s="1" t="n"/>
+      <c r="O4" s="1" t="n"/>
+      <c r="P4" s="1" t="n"/>
+      <c r="Q4" s="1" t="n"/>
+    </row>
+    <row r="5" ht="15" customHeight="1" thickBot="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total </t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Amount Total</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Amount Division</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="n"/>
+      <c r="G5" s="1" t="n"/>
+      <c r="H5" s="1" t="n"/>
+      <c r="I5" s="1" t="n"/>
+      <c r="J5" s="1" t="n"/>
+      <c r="K5" s="1" t="n"/>
+      <c r="L5" s="1" t="n"/>
+      <c r="M5" s="1" t="n"/>
+      <c r="N5" s="1" t="n"/>
+      <c r="O5" s="1" t="n"/>
+      <c r="P5" s="1" t="n"/>
+      <c r="Q5" s="1" t="n"/>
+    </row>
+    <row r="6" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Total:</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>1.- Equity (to be injected in year 0)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="1" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="1" t="n"/>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="n"/>
+      <c r="O6" s="1" t="n"/>
+      <c r="P6" s="1" t="n"/>
+      <c r="Q6" s="1" t="n"/>
+    </row>
+    <row r="7" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Total:</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>2.- Grants (inyected in the first two years but linked to CAPEX deployment)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="1" t="n"/>
+      <c r="G7" s="1" t="n"/>
+      <c r="H7" s="1" t="n"/>
+      <c r="I7" s="1" t="n"/>
+      <c r="J7" s="1" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="1" t="n"/>
+      <c r="M7" s="1" t="n"/>
+      <c r="N7" s="1" t="n"/>
+      <c r="O7" s="1" t="n"/>
+      <c r="P7" s="1" t="n"/>
+      <c r="Q7" s="1" t="n"/>
+    </row>
+    <row r="8" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Total:</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>3.- Debt</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="n"/>
+      <c r="H8" s="1" t="n"/>
+      <c r="I8" s="1" t="n"/>
+      <c r="J8" s="1" t="n"/>
+      <c r="K8" s="1" t="n"/>
+      <c r="L8" s="1" t="n"/>
+      <c r="M8" s="1" t="n"/>
+      <c r="N8" s="1" t="n"/>
+      <c r="O8" s="1" t="n"/>
+      <c r="P8" s="1" t="n"/>
+      <c r="Q8" s="1" t="n"/>
+    </row>
+    <row r="9" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="1" t="n"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Interests</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="1" t="n"/>
+      <c r="G9" s="1" t="n"/>
+      <c r="H9" s="1" t="n"/>
+      <c r="I9" s="1" t="n"/>
+      <c r="J9" s="1" t="n"/>
+      <c r="K9" s="1" t="n"/>
+      <c r="L9" s="1" t="n"/>
+      <c r="M9" s="1" t="n"/>
+      <c r="N9" s="1" t="n"/>
+      <c r="O9" s="1" t="n"/>
+      <c r="P9" s="1" t="n"/>
+      <c r="Q9" s="1" t="n"/>
+    </row>
+    <row r="10" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Grace period</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="n"/>
+      <c r="H10" s="1" t="n"/>
+      <c r="I10" s="1" t="n"/>
+      <c r="J10" s="1" t="n"/>
+      <c r="K10" s="1" t="n"/>
+      <c r="L10" s="1" t="n"/>
+      <c r="M10" s="1" t="n"/>
+      <c r="N10" s="1" t="n"/>
+      <c r="O10" s="1" t="n"/>
+      <c r="P10" s="1" t="n"/>
+      <c r="Q10" s="1" t="n"/>
+    </row>
+    <row r="11" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Amortization period</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
+      <c r="H11" s="1" t="n"/>
+      <c r="I11" s="1" t="n"/>
+      <c r="J11" s="1" t="n"/>
+      <c r="K11" s="1" t="n"/>
+      <c r="L11" s="1" t="n"/>
+      <c r="M11" s="1" t="n"/>
+      <c r="N11" s="1" t="n"/>
+      <c r="O11" s="1" t="n"/>
+      <c r="P11" s="1" t="n"/>
+      <c r="Q11" s="1" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="1" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
+      <c r="H12" s="1" t="n"/>
+      <c r="I12" s="1" t="n"/>
+      <c r="J12" s="1" t="n"/>
+      <c r="K12" s="1" t="n"/>
+      <c r="L12" s="1" t="n"/>
+      <c r="M12" s="1" t="n"/>
+      <c r="N12" s="1" t="n"/>
+      <c r="O12" s="1" t="n"/>
+      <c r="P12" s="1" t="n"/>
+      <c r="Q12" s="1" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>2025</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>2026</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>2027</v>
+      </c>
+      <c r="K13" s="9" t="n">
+        <v>2028</v>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>2029</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>2030</v>
+      </c>
+      <c r="N13" s="9" t="n">
+        <v>2031</v>
+      </c>
+      <c r="O13" s="9" t="n">
+        <v>2032</v>
+      </c>
+      <c r="P13" s="9" t="n">
+        <v>2033</v>
+      </c>
+      <c r="Q13" s="9" t="n">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="14" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="1" t="n"/>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Annual debt needs</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n"/>
+      <c r="E14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!F22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="F14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!F22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="G14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!G22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="H14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!H22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="I14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!I22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="J14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!J22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="K14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!K22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="L14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!L22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="M14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!M22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="N14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!N22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="O14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!O22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="P14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!P22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+      <c r="Q14" s="11">
+        <f>IF('[1]CleanStep - JUSTACCESS - FFSS'!Q22&gt;0,"ok","increase debt")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1" thickBot="1" thickTop="1">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="1" t="n"/>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>How much to increase</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="1" t="n"/>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Debt increase</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>M$</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="13" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C14:AJ14">

</xml_diff>